<commit_message>
Ch 6 Week 2 Second Revision
</commit_message>
<xml_diff>
--- a/Figures & Tables/Chapter 6/Table 1 - Codebook for the Bi-Weekly Reports.xlsx
+++ b/Figures & Tables/Chapter 6/Table 1 - Codebook for the Bi-Weekly Reports.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\github\Thesis-Document\Figures &amp; Tables\Chapter 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB388A7-7E12-4C06-ABFA-75534E3AB836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7526AE1E-6820-4E4E-A9F9-C46C5AD6450A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C203C5F8-6440-45F2-83B8-D5A158C4B652}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C203C5F8-6440-45F2-83B8-D5A158C4B652}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
   <si>
     <t>Category</t>
   </si>
@@ -213,13 +214,103 @@
   </si>
   <si>
     <t>The group reports that they are giving up on reaching someone and they are working with the available resources</t>
+  </si>
+  <si>
+    <t>Team A</t>
+  </si>
+  <si>
+    <t>Team B</t>
+  </si>
+  <si>
+    <t>Team C</t>
+  </si>
+  <si>
+    <t>Team D</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>WorkshopAR</t>
+  </si>
+  <si>
+    <t>For the week</t>
+  </si>
+  <si>
+    <t>For the assigment</t>
+  </si>
+  <si>
+    <t>Planification</t>
+  </si>
+  <si>
+    <t>Progress</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Consolidation</t>
+  </si>
+  <si>
+    <t>Structure</t>
+  </si>
+  <si>
+    <t>Communication</t>
+  </si>
+  <si>
+    <t>Architectural Desing</t>
+  </si>
+  <si>
+    <t>Material Decisions</t>
+  </si>
+  <si>
+    <t>Cost Estimation</t>
+  </si>
+  <si>
+    <t>Poster</t>
+  </si>
+  <si>
+    <t>Meetings</t>
+  </si>
+  <si>
+    <t>Responsabilities</t>
+  </si>
+  <si>
+    <t>Infromation Needed</t>
+  </si>
+  <si>
+    <t>Doing good</t>
+  </si>
+  <si>
+    <t>Can help a lot</t>
+  </si>
+  <si>
+    <t>Doing Okay</t>
+  </si>
+  <si>
+    <t>May be of help</t>
+  </si>
+  <si>
+    <t>Could be better</t>
+  </si>
+  <si>
+    <t>Not very helpful</t>
+  </si>
+  <si>
+    <t>Doing bad</t>
+  </si>
+  <si>
+    <t>Not helpful</t>
+  </si>
+  <si>
+    <t>No data</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,16 +331,54 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -293,11 +422,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right style="medium">
+        <color theme="0"/>
+      </right>
+      <top style="medium">
+        <color theme="0"/>
+      </top>
+      <bottom style="medium">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -308,16 +461,63 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -678,7 +878,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2">
@@ -692,7 +892,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
+      <c r="A3" s="5"/>
       <c r="B3" s="2">
         <v>1.2</v>
       </c>
@@ -704,7 +904,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
+      <c r="A4" s="5"/>
       <c r="B4" s="2">
         <v>1.3</v>
       </c>
@@ -716,7 +916,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
+      <c r="A5" s="5"/>
       <c r="B5" s="2">
         <v>1.4</v>
       </c>
@@ -740,7 +940,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="2">
@@ -754,7 +954,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4"/>
+      <c r="A8" s="5"/>
       <c r="B8" s="2">
         <v>2.2000000000000002</v>
       </c>
@@ -778,7 +978,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="2">
@@ -792,7 +992,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4"/>
+      <c r="A11" s="5"/>
       <c r="B11" s="2">
         <v>3.2</v>
       </c>
@@ -804,7 +1004,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
+      <c r="A12" s="5"/>
       <c r="B12" s="2">
         <v>3.3</v>
       </c>
@@ -816,7 +1016,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4"/>
+      <c r="A13" s="5"/>
       <c r="B13" s="2">
         <v>3.4</v>
       </c>
@@ -840,7 +1040,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="2">
@@ -854,7 +1054,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4"/>
+      <c r="A16" s="5"/>
       <c r="B16" s="2">
         <v>4.2</v>
       </c>
@@ -866,7 +1066,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4"/>
+      <c r="A17" s="5"/>
       <c r="B17" s="2">
         <v>4.3</v>
       </c>
@@ -878,7 +1078,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4"/>
+      <c r="A18" s="5"/>
       <c r="B18" s="2">
         <v>4.4000000000000004</v>
       </c>
@@ -890,7 +1090,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4"/>
+      <c r="A19" s="5"/>
       <c r="B19" s="2">
         <v>4.5</v>
       </c>
@@ -902,7 +1102,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4"/>
+      <c r="A20" s="5"/>
       <c r="B20" s="2">
         <v>4.5999999999999996</v>
       </c>
@@ -926,7 +1126,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B22" s="2">
@@ -940,7 +1140,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="4"/>
+      <c r="A23" s="5"/>
       <c r="B23" s="2">
         <v>5.2</v>
       </c>
@@ -952,7 +1152,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="4"/>
+      <c r="A24" s="5"/>
       <c r="B24" s="2">
         <v>5.3</v>
       </c>
@@ -964,7 +1164,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4"/>
+      <c r="A25" s="5"/>
       <c r="B25" s="2">
         <v>5.4</v>
       </c>
@@ -997,4 +1197,294 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A68EE7-CFF7-416F-B0CC-B0538A7A55CB}">
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="10" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="9"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="10"/>
+      <c r="E1" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" s="11"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="22"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="25"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
+      <c r="B4" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="22"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="22"/>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="25"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="25"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="25"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="24"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="25"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13"/>
+      <c r="B9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="25"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="25"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="26"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13"/>
+      <c r="B13" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="18"/>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13"/>
+      <c r="B14" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="19"/>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="C16" s="15"/>
+      <c r="D16" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="17"/>
+      <c r="F16" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="G16" s="18"/>
+      <c r="H16" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="19"/>
+      <c r="J16" s="20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="3:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="C17" s="15"/>
+      <c r="D17" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" s="17"/>
+      <c r="F17" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" s="18"/>
+      <c r="H17" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="19"/>
+      <c r="J17" s="16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="F19" s="21"/>
+      <c r="G19" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A6:A10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>